<commit_message>
Verifica settimanale: 149 duplicati cross-file marcati (deduplica globale)
Deduplica globale su tutti i file .xlsx in /output (ragione_sociale
normalizzata + dominio sito_web). Le occorrenze duplicate sono annotate
in nota con riferimento al file canonico (occorrenza più vecchia), senza
toccare le righe canoniche né cancellare dati. Il doppio controllo
WebSearch sui record "DA VERIFICARE UMANAMENTE" dei file nuovi è in corso
in background e sarà incluso in un commit successivo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Cdg7xAX5zjFFAvDY4pLGt
</commit_message>
<xml_diff>
--- a/output/2026-09-03_18_Italia_Basilicata_Depolverazione_Trattamento_aria.xlsx
+++ b/output/2026-09-03_18_Italia_Basilicata_Depolverazione_Trattamento_aria.xlsx
@@ -498,10 +498,9 @@
           <t>0835 264263 / 392 9823056</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Azienda confermata attiva da oltre 30 anni nella vendita di macchine e attrezzature per pulizia industriale, tra cui aspiraliquidi, aspiratori industriali, compressori, generatori aria calda, idropulitrici, spazzatrici. Sede: Contrada Serra Paducci, Zona Commerciale 2, 75100 Matera (MT). Distribuzione estesa a Puglia e Basilicata. Email generica non reperita.</t>
+          <t>Azienda confermata attiva da oltre 30 anni nella vendita di macchine e attrezzature per pulizia industriale, tra cui aspiraliquidi, aspiratori industriali, compressori, generatori aria calda, idropulitrici, spazzatrici. Sede: Contrada Serra Paducci, Zona Commerciale 2, 75100 Matera (MT). Distribuzione estesa a Puglia e Basilicata. Email generica non reperita. [DUPLICATO — vedi anche: 2026-09-03_17_Italia_Basilicata_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -543,7 +542,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Azienda confermata, attiva da 25 anni nella vendita di macchine e attrezzature per pulizia industriale (aspiratori, idropulitrici, lavapavimenti, spazzatrici, lavamoquette). Operativa a Matera e in Basilicata/Puglia. Indirizzo esatto non reperito nelle fonti consultate (solo 'Matera, MT').</t>
+          <t>Azienda confermata, attiva da 25 anni nella vendita di macchine e attrezzature per pulizia industriale (aspiratori, idropulitrici, lavapavimenti, spazzatrici, lavamoquette). Operativa a Matera e in Basilicata/Puglia. Indirizzo esatto non reperito nelle fonti consultate (solo 'Matera, MT'). [DUPLICATO — vedi anche: 2026-09-03_17_Italia_Basilicata_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">

</xml_diff>